<commit_message>
IF, MIN, MAX, ABS, ROUND, README ve GitHub Actions
</commit_message>
<xml_diff>
--- a/examples/kar_modeli.xlsx
+++ b/examples/kar_modeli.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Kar Modeli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kar Modeli" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -539,6 +539,28 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Vergi</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>MAX(0, B13)*0.2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Net kâr</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>B13-B14</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>